<commit_message>
Grant run 2026-10-12: add three county opioid settlement programs
Advances last week's lead into concrete pipeline entries.

Somerset County micro-grants enter at 40%, third on the board and the
best structural fit found anywhere in this project: 501(c)(3)-only,
one-county applicant pool, application is a statement of interest plus a
budget, and at least $450k/year recurring for 18 years. It inverts every
constraint that sank the September items.

Union County enters at 30% - roughly $17.7M over 18 years for recovery
support, treatment, early intervention and harm reduction, with cycles
running late winter. Morris County at 20%.

No Essex County program surfaced; the state's $10.5M Essex allocation is
state-administered. Pipeline now holds 30 scored rows, and for the first
time these cycles sit ahead of the organization rather than behind it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CptqzmsujXJyvXahcJxHJY
</commit_message>
<xml_diff>
--- a/grant_search/data/grant_pipeline.xlsx
+++ b/grant_search/data/grant_pipeline.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Method" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline'!$A$4:$Q$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pipeline'!$A$4:$Q$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -605,7 +605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q35"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -869,25 +869,23 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Empowerment Grant</t>
+          <t>Opioid Settlement micro-grants</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Provident Bank Foundation</t>
+          <t>Somerset County Human Services</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Private foundation</t>
-        </is>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>46507</v>
-      </c>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n"/>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Next cycle ~early 2027</t>
         </is>
       </c>
       <c r="G7" s="7">
@@ -898,14 +896,14 @@
         <v>5000</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="J7" s="11">
         <f>IF(AND(H7&lt;&gt;"",I7&lt;&gt;""),AVERAGE(H7:I7),IF(I7&lt;&gt;"",I7*$C$3,IF(H7&lt;&gt;"",H7,"")))</f>
         <v/>
       </c>
       <c r="K7" s="12" t="n">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="L7" s="11">
         <f>IF(OR(J7="",K7=""),"",J7*K7)</f>
@@ -921,7 +919,7 @@
       <c r="P7" s="14" t="n"/>
       <c r="Q7" s="8" t="inlineStr">
         <is>
-          <t>CRA-driven giving favors local community orgs. Award size fits budget.</t>
+          <t>STRONGEST STRUCTURAL FIT FOUND. 501(c)(3)-only, one-county applicant pool, award sized to the org, application is a statement of interest plus budget. Funded by the county's opioid settlement share - at least $450k/year for 18 years, so a missed cycle is a delay not a loss. Somerset is a priority county.</t>
         </is>
       </c>
     </row>
@@ -931,21 +929,21 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Project ATLAS</t>
+          <t>Empowerment Grant</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of State, Office of Faith Based Initiatives</t>
+          <t>Provident Bank Foundation</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E8" s="15" t="n">
-        <v>46444</v>
+        <v>46507</v>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
@@ -956,9 +954,11 @@
         <f>IF(E8="","",E8-TODAY())</f>
         <v/>
       </c>
-      <c r="H8" s="10" t="n"/>
+      <c r="H8" s="10" t="n">
+        <v>5000</v>
+      </c>
       <c r="I8" s="10" t="n">
-        <v>10000</v>
+        <v>25000</v>
       </c>
       <c r="J8" s="11">
         <f>IF(AND(H8&lt;&gt;"",I8&lt;&gt;""),AVERAGE(H8:I8),IF(I8&lt;&gt;"",I8*$C$3,IF(H8&lt;&gt;"",H8,"")))</f>
@@ -981,7 +981,7 @@
       <c r="P8" s="14" t="n"/>
       <c r="Q8" s="8" t="inlineStr">
         <is>
-          <t>State office that exists to fund grassroots community work.</t>
+          <t>CRA-driven giving favors local community orgs. Award size fits budget.</t>
         </is>
       </c>
     </row>
@@ -991,25 +991,25 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>General Operating and Project Grants</t>
+          <t>Project ATLAS</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Partners For Health Foundation</t>
+          <t>NJ Dept. of State, Office of Faith Based Initiatives</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Private foundation</t>
+          <t>State / regional</t>
         </is>
       </c>
       <c r="E9" s="15" t="n">
-        <v>46441</v>
+        <v>46444</v>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Pre-proposal</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G9" s="7">
@@ -1017,21 +1017,23 @@
         <v/>
       </c>
       <c r="H9" s="10" t="n"/>
-      <c r="I9" s="10" t="n"/>
+      <c r="I9" s="10" t="n">
+        <v>10000</v>
+      </c>
       <c r="J9" s="11">
         <f>IF(AND(H9&lt;&gt;"",I9&lt;&gt;""),AVERAGE(H9:I9),IF(I9&lt;&gt;"",I9*$C$3,IF(H9&lt;&gt;"",H9,"")))</f>
         <v/>
       </c>
       <c r="K9" s="12" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="L9" s="11">
         <f>IF(OR(J9="",K9=""),"",J9*K9)</f>
         <v/>
       </c>
-      <c r="M9" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="N9" s="14" t="n"/>
@@ -1039,7 +1041,7 @@
       <c r="P9" s="14" t="n"/>
       <c r="Q9" s="8" t="inlineStr">
         <is>
-          <t>Essex County health funder. GENERAL OPERATING support - rare and worth more per dollar than restricted money. Amount unpublished; confirm range. Verify the org sits inside its service footprint.</t>
+          <t>State office that exists to fund grassroots community work.</t>
         </is>
       </c>
     </row>
@@ -1049,12 +1051,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Standard Grants</t>
+          <t>General Operating and Project Grants</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Healthcare Foundation of New Jersey</t>
+          <t>Partners For Health Foundation</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -1063,27 +1065,25 @@
         </is>
       </c>
       <c r="E10" s="15" t="n">
-        <v>46345</v>
+        <v>46441</v>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Pre-proposal</t>
         </is>
       </c>
       <c r="G10" s="7">
         <f>IF(E10="","",E10-TODAY())</f>
         <v/>
       </c>
-      <c r="H10" s="10" t="n">
-        <v>35000</v>
-      </c>
+      <c r="H10" s="10" t="n"/>
       <c r="I10" s="10" t="n"/>
       <c r="J10" s="11">
         <f>IF(AND(H10&lt;&gt;"",I10&lt;&gt;""),AVERAGE(H10:I10),IF(I10&lt;&gt;"",I10*$C$3,IF(H10&lt;&gt;"",H10,"")))</f>
         <v/>
       </c>
       <c r="K10" s="12" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="L10" s="11">
         <f>IF(OR(J10="",K10=""),"",J10*K10)</f>
@@ -1099,7 +1099,7 @@
       <c r="P10" s="14" t="n"/>
       <c r="Q10" s="8" t="inlineStr">
         <is>
-          <t>3 of 4 priority counties in footprint; reported behavioral health emphasis. OPEN QUESTION: does a non-Federation-affiliated org qualify under the 'vulnerable populations elsewhere in Essex, Morris, Union' clause?</t>
+          <t>Essex County health funder. GENERAL OPERATING support - rare and worth more per dollar than restricted money. Amount unpublished; confirm range. Verify the org sits inside its service footprint.</t>
         </is>
       </c>
     </row>
@@ -1109,51 +1109,47 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Empower New Jersey Grant</t>
+          <t>Opioid Settlement Funds annual RFA</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Community Foundation of New Jersey</t>
+          <t>Union County OBHSM</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Private foundation</t>
-        </is>
-      </c>
-      <c r="E11" s="15" t="n">
-        <v>46295</v>
-      </c>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n"/>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Next cycle ~early 2027</t>
         </is>
       </c>
       <c r="G11" s="7">
         <f>IF(E11="","",E11-TODAY())</f>
         <v/>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="10" t="n"/>
+      <c r="I11" s="10" t="n">
         <v>50000</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <v>100000</v>
       </c>
       <c r="J11" s="11">
         <f>IF(AND(H11&lt;&gt;"",I11&lt;&gt;""),AVERAGE(H11:I11),IF(I11&lt;&gt;"",I11*$C$3,IF(H11&lt;&gt;"",H11,"")))</f>
         <v/>
       </c>
       <c r="K11" s="12" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="L11" s="11">
         <f>IF(OR(J11="",K11=""),"",J11*K11)</f>
         <v/>
       </c>
-      <c r="M11" s="16" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="N11" s="14" t="n"/>
@@ -1161,7 +1157,7 @@
       <c r="P11" s="14" t="n"/>
       <c r="Q11" s="8" t="inlineStr">
         <is>
-          <t>Best effort-to-return balance on the list. If only one thing gets written this fall, this is it.</t>
+          <t>Union County holds ~$17.7M over 18 years (~$980k/yr) for recovery support, treatment, early intervention and harm reduction. RFA 2026-059 closed 2026-03-18, so cycles run late winter. Priority county; a durable relationship rather than a one-off.</t>
         </is>
       </c>
     </row>
@@ -1171,21 +1167,21 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>VAWA Competitive Grant Program</t>
+          <t>Standard Grants</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Law &amp; Public Safety</t>
+          <t>Healthcare Foundation of New Jersey</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E12" s="15" t="n">
-        <v>46553</v>
+        <v>46345</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
@@ -1196,16 +1192,16 @@
         <f>IF(E12="","",E12-TODAY())</f>
         <v/>
       </c>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="10" t="n">
-        <v>75000</v>
-      </c>
+      <c r="H12" s="10" t="n">
+        <v>35000</v>
+      </c>
+      <c r="I12" s="10" t="n"/>
       <c r="J12" s="11">
         <f>IF(AND(H12&lt;&gt;"",I12&lt;&gt;""),AVERAGE(H12:I12),IF(I12&lt;&gt;"",I12*$C$3,IF(H12&lt;&gt;"",H12,"")))</f>
         <v/>
       </c>
       <c r="K12" s="12" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="L12" s="11">
         <f>IF(OR(J12="",K12=""),"",J12*K12)</f>
@@ -1221,7 +1217,7 @@
       <c r="P12" s="14" t="n"/>
       <c r="Q12" s="8" t="inlineStr">
         <is>
-          <t>Maps onto stated DV prevention work. Will want demonstrated DV programming, not just adjacent capacity.</t>
+          <t>3 of 4 priority counties in footprint; reported behavioral health emphasis. OPEN QUESTION: does a non-Federation-affiliated org qualify under the 'vulnerable populations elsewhere in Essex, Morris, Union' clause?</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1227,12 @@
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Awards for Advancing Minority Mental Health</t>
+          <t>Empower New Jersey Grant</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>American Psychiatric Association Foundation</t>
+          <t>Community Foundation of New Jersey</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -1245,7 +1241,7 @@
         </is>
       </c>
       <c r="E13" s="15" t="n">
-        <v>46418</v>
+        <v>46295</v>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
@@ -1257,10 +1253,10 @@
         <v/>
       </c>
       <c r="H13" s="10" t="n">
-        <v>5000</v>
+        <v>50000</v>
       </c>
       <c r="I13" s="10" t="n">
-        <v>5000</v>
+        <v>100000</v>
       </c>
       <c r="J13" s="11">
         <f>IF(AND(H13&lt;&gt;"",I13&lt;&gt;""),AVERAGE(H13:I13),IF(I13&lt;&gt;"",I13*$C$3,IF(H13&lt;&gt;"",H13,"")))</f>
@@ -1283,7 +1279,7 @@
       <c r="P13" s="14" t="n"/>
       <c r="Q13" s="8" t="inlineStr">
         <is>
-          <t>National pool but tiny award. Real value is the credential, not the cash.</t>
+          <t>Best effort-to-return balance on the list. If only one thing gets written this fall, this is it.</t>
         </is>
       </c>
     </row>
@@ -1293,21 +1289,21 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Champions in Action</t>
+          <t>VAWA Competitive Grant Program</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Citizens Charitable Foundation</t>
+          <t>NJ Dept. of Law &amp; Public Safety</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Private foundation</t>
+          <t>State / regional</t>
         </is>
       </c>
       <c r="E14" s="15" t="n">
-        <v>46295</v>
+        <v>46553</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -1318,18 +1314,16 @@
         <f>IF(E14="","",E14-TODAY())</f>
         <v/>
       </c>
-      <c r="H14" s="10" t="n">
-        <v>50000</v>
-      </c>
+      <c r="H14" s="10" t="n"/>
       <c r="I14" s="10" t="n">
-        <v>50000</v>
+        <v>75000</v>
       </c>
       <c r="J14" s="11">
         <f>IF(AND(H14&lt;&gt;"",I14&lt;&gt;""),AVERAGE(H14:I14),IF(I14&lt;&gt;"",I14*$C$3,IF(H14&lt;&gt;"",H14,"")))</f>
         <v/>
       </c>
       <c r="K14" s="12" t="n">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="L14" s="11">
         <f>IF(OR(J14="",K14=""),"",J14*K14)</f>
@@ -1345,7 +1339,7 @@
       <c r="P14" s="14" t="n"/>
       <c r="Q14" s="8" t="inlineStr">
         <is>
-          <t>UPGRADED 2026-08-23. Budget eligibility confirmed ($250k-$5M; the org qualifies). 2026 theme 'Uplifting Resilient Nonprofits' is broad and favourable. Award is $50k plus volunteer engagement and promotion. CATCH: applicants must host 1-2 volunteer projects for Citizens staff, at least one skills-based - needs a credible plan given client confidentiality.</t>
+          <t>Maps onto stated DV prevention work. Will want demonstrated DV programming, not just adjacent capacity.</t>
         </is>
       </c>
     </row>
@@ -1355,49 +1349,51 @@
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Pathways to Recovery - Round 2 NGO</t>
+          <t>Awards for Advancing Minority Mental Health</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
+          <t>American Psychiatric Association Foundation</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E15" s="15" t="n">
-        <v>46472</v>
+        <v>46418</v>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>LOI</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G15" s="7">
         <f>IF(E15="","",E15-TODAY())</f>
         <v/>
       </c>
-      <c r="H15" s="10" t="n"/>
+      <c r="H15" s="10" t="n">
+        <v>5000</v>
+      </c>
       <c r="I15" s="10" t="n">
-        <v>1000000</v>
+        <v>5000</v>
       </c>
       <c r="J15" s="11">
         <f>IF(AND(H15&lt;&gt;"",I15&lt;&gt;""),AVERAGE(H15:I15),IF(I15&lt;&gt;"",I15*$C$3,IF(H15&lt;&gt;"",H15,"")))</f>
         <v/>
       </c>
       <c r="K15" s="12" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="L15" s="11">
         <f>IF(OR(J15="",K15=""),"",J15*K15)</f>
         <v/>
       </c>
-      <c r="M15" s="17" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="M15" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="N15" s="14" t="n"/>
@@ -1405,7 +1401,7 @@
       <c r="P15" s="14" t="n"/>
       <c r="Q15" s="8" t="inlineStr">
         <is>
-          <t>HIGHEST EXPECTED VALUE on the list. NJ-only pool, NGO-specific track, opioid focus matches directly. Ask well under the cap.</t>
+          <t>National pool but tiny award. Real value is the credential, not the cash.</t>
         </is>
       </c>
     </row>
@@ -1415,12 +1411,12 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Pathways to Recovery (general)</t>
+          <t>Opioid Settlement priorities</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
+          <t>Morris County Human Services</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
@@ -1428,36 +1424,34 @@
           <t>State / regional</t>
         </is>
       </c>
-      <c r="E16" s="15" t="n">
-        <v>46451</v>
-      </c>
+      <c r="E16" s="7" t="n"/>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>LOI</t>
+          <t>Confirm cycle</t>
         </is>
       </c>
       <c r="G16" s="7">
         <f>IF(E16="","",E16-TODAY())</f>
         <v/>
       </c>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="10" t="n">
-        <v>1000000</v>
-      </c>
+      <c r="H16" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I16" s="10" t="n"/>
       <c r="J16" s="11">
         <f>IF(AND(H16&lt;&gt;"",I16&lt;&gt;""),AVERAGE(H16:I16),IF(I16&lt;&gt;"",I16*$C$3,IF(H16&lt;&gt;"",H16,"")))</f>
         <v/>
       </c>
       <c r="K16" s="12" t="n">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="L16" s="11">
         <f>IF(OR(J16="",K16=""),"",J16*K16)</f>
         <v/>
       </c>
-      <c r="M16" s="17" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="M16" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="N16" s="14" t="n"/>
@@ -1465,7 +1459,7 @@
       <c r="P16" s="14" t="n"/>
       <c r="Q16" s="8" t="inlineStr">
         <is>
-          <t>Same program, broader applicant pool than the NGO track.</t>
+          <t>Minimum request $5,000. Morris is outside the four priority counties but inside HFNJ's Greater MetroWest footprint, so already adjacent to the org's reach.</t>
         </is>
       </c>
     </row>
@@ -1475,49 +1469,51 @@
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Specific Population Community Grant</t>
+          <t>Champions in Action</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Health</t>
+          <t>Citizens Charitable Foundation</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E17" s="15" t="n">
-        <v>46525</v>
+        <v>46295</v>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>LOI</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G17" s="7">
         <f>IF(E17="","",E17-TODAY())</f>
         <v/>
       </c>
-      <c r="H17" s="10" t="n"/>
+      <c r="H17" s="10" t="n">
+        <v>50000</v>
+      </c>
       <c r="I17" s="10" t="n">
-        <v>500000</v>
+        <v>50000</v>
       </c>
       <c r="J17" s="11">
         <f>IF(AND(H17&lt;&gt;"",I17&lt;&gt;""),AVERAGE(H17:I17),IF(I17&lt;&gt;"",I17*$C$3,IF(H17&lt;&gt;"",H17,"")))</f>
         <v/>
       </c>
       <c r="K17" s="12" t="n">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="L17" s="11">
         <f>IF(OR(J17="",K17=""),"",J17*K17)</f>
         <v/>
       </c>
-      <c r="M17" s="17" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="M17" s="16" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="N17" s="14" t="n"/>
@@ -1525,7 +1521,7 @@
       <c r="P17" s="14" t="n"/>
       <c r="Q17" s="8" t="inlineStr">
         <is>
-          <t>Justice-involved qualifies as a specific population. Award size demands strong fiscal infrastructure.</t>
+          <t>UPGRADED 2026-08-23. Budget eligibility confirmed ($250k-$5M; the org qualifies). 2026 theme 'Uplifting Resilient Nonprofits' is broad and favourable. Award is $50k plus volunteer engagement and promotion. CATCH: applicants must host 1-2 volunteer projects for Citizens staff, at least one skills-based - needs a credible plan given client confidentiality.</t>
         </is>
       </c>
     </row>
@@ -1535,25 +1531,25 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Therapeutic Giving: Neuroscience - Local &amp; Regional</t>
+          <t>Pathways to Recovery - Round 2 NGO</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Johnson &amp; Johnson Innovative Medicine</t>
+          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Private foundation</t>
+          <t>State / regional</t>
         </is>
       </c>
       <c r="E18" s="15" t="n">
-        <v>46538</v>
+        <v>46472</v>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>LOI</t>
         </is>
       </c>
       <c r="G18" s="7">
@@ -1561,13 +1557,15 @@
         <v/>
       </c>
       <c r="H18" s="10" t="n"/>
-      <c r="I18" s="10" t="n"/>
+      <c r="I18" s="10" t="n">
+        <v>1000000</v>
+      </c>
       <c r="J18" s="11">
         <f>IF(AND(H18&lt;&gt;"",I18&lt;&gt;""),AVERAGE(H18:I18),IF(I18&lt;&gt;"",I18*$C$3,IF(H18&lt;&gt;"",H18,"")))</f>
         <v/>
       </c>
       <c r="K18" s="12" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="L18" s="11">
         <f>IF(OR(J18="",K18=""),"",J18*K18)</f>
@@ -1583,7 +1581,7 @@
       <c r="P18" s="14" t="n"/>
       <c r="Q18" s="8" t="inlineStr">
         <is>
-          <t>Corporate giving with a local/regional track; mental health sits under its neuroscience umbrella. Pharma giving tends to favor established orgs and clinically-adjacent work, which caps the odds. Amount unpublished.</t>
+          <t>HIGHEST EXPECTED VALUE on the list. NJ-only pool, NGO-specific track, opioid focus matches directly. Ask well under the cap.</t>
         </is>
       </c>
     </row>
@@ -1593,25 +1591,25 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>Citizens Philanthropic Foundation: Workforce Development</t>
+          <t>Pathways to Recovery (general)</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>Citizens Philanthropic Foundation</t>
+          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Private foundation</t>
+          <t>State / regional</t>
         </is>
       </c>
       <c r="E19" s="15" t="n">
-        <v>46529</v>
+        <v>46451</v>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>LOI</t>
         </is>
       </c>
       <c r="G19" s="7">
@@ -1619,7 +1617,9 @@
         <v/>
       </c>
       <c r="H19" s="10" t="n"/>
-      <c r="I19" s="10" t="n"/>
+      <c r="I19" s="10" t="n">
+        <v>1000000</v>
+      </c>
       <c r="J19" s="11">
         <f>IF(AND(H19&lt;&gt;"",I19&lt;&gt;""),AVERAGE(H19:I19),IF(I19&lt;&gt;"",I19*$C$3,IF(H19&lt;&gt;"",H19,"")))</f>
         <v/>
@@ -1641,7 +1641,7 @@
       <c r="P19" s="14" t="n"/>
       <c r="Q19" s="8" t="inlineStr">
         <is>
-          <t>Reentry employment is a workable framing. Note this is the same corporate family as Champions in Action - a relationship built through one may help the other. Amount unpublished.</t>
+          <t>Same program, broader applicant pool than the NGO track.</t>
         </is>
       </c>
     </row>
@@ -1651,12 +1651,12 @@
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Job Opportunities for Building Success</t>
+          <t>Specific Population Community Grant</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
+          <t>NJ Dept. of Health</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="E20" s="15" t="n">
-        <v>46450</v>
+        <v>46525</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
@@ -1678,14 +1678,14 @@
       </c>
       <c r="H20" s="10" t="n"/>
       <c r="I20" s="10" t="n">
-        <v>1000000</v>
+        <v>500000</v>
       </c>
       <c r="J20" s="11">
         <f>IF(AND(H20&lt;&gt;"",I20&lt;&gt;""),AVERAGE(H20:I20),IF(I20&lt;&gt;"",I20*$C$3,IF(H20&lt;&gt;"",H20,"")))</f>
         <v/>
       </c>
       <c r="K20" s="12" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="L20" s="11">
         <f>IF(OR(J20="",K20=""),"",J20*K20)</f>
@@ -1701,7 +1701,7 @@
       <c r="P20" s="14" t="n"/>
       <c r="Q20" s="8" t="inlineStr">
         <is>
-          <t>Reentry employment framing works, but competitors are established workforce development agencies.</t>
+          <t>Justice-involved qualifies as a specific population. Award size demands strong fiscal infrastructure.</t>
         </is>
       </c>
     </row>
@@ -1711,12 +1711,12 @@
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Family foundations (Scripps, Kim/Kayasa, Bernau, Scaife)</t>
+          <t>Therapeutic Giving: Neuroscience - Local &amp; Regional</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Various</t>
+          <t>Johnson &amp; Johnson Innovative Medicine</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -1724,10 +1724,12 @@
           <t>Private foundation</t>
         </is>
       </c>
-      <c r="E21" s="7" t="n"/>
+      <c r="E21" s="15" t="n">
+        <v>46538</v>
+      </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Rolling / 2027</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G21" s="7">
@@ -1741,15 +1743,15 @@
         <v/>
       </c>
       <c r="K21" s="12" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="L21" s="11">
         <f>IF(OR(J21="",K21=""),"",J21*K21)</f>
         <v/>
       </c>
-      <c r="M21" s="18" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="M21" s="17" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="N21" s="14" t="n"/>
@@ -1757,7 +1759,7 @@
       <c r="P21" s="14" t="n"/>
       <c r="Q21" s="8" t="inlineStr">
         <is>
-          <t>Priorities unpublished; many small family foundations are effectively invitation-only. Pull Form 990s before writing - 15 min each tells you whether they accept unsolicited requests at all.</t>
+          <t>Corporate giving with a local/regional track; mental health sits under its neuroscience umbrella. Pharma giving tends to favor established orgs and clinically-adjacent work, which caps the odds. Amount unpublished.</t>
         </is>
       </c>
     </row>
@@ -1767,12 +1769,12 @@
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Get Out and Get Active Grant</t>
+          <t>Citizens Philanthropic Foundation: Workforce Development</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>Anxiety &amp; Depression Initiative</t>
+          <t>Citizens Philanthropic Foundation</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
@@ -1781,7 +1783,7 @@
         </is>
       </c>
       <c r="E22" s="15" t="n">
-        <v>46504</v>
+        <v>46529</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
@@ -1793,15 +1795,13 @@
         <v/>
       </c>
       <c r="H22" s="10" t="n"/>
-      <c r="I22" s="10" t="n">
-        <v>10000</v>
-      </c>
+      <c r="I22" s="10" t="n"/>
       <c r="J22" s="11">
         <f>IF(AND(H22&lt;&gt;"",I22&lt;&gt;""),AVERAGE(H22:I22),IF(I22&lt;&gt;"",I22*$C$3,IF(H22&lt;&gt;"",H22,"")))</f>
         <v/>
       </c>
       <c r="K22" s="12" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="L22" s="11">
         <f>IF(OR(J22="",K22=""),"",J22*K22)</f>
@@ -1817,7 +1817,7 @@
       <c r="P22" s="14" t="n"/>
       <c r="Q22" s="8" t="inlineStr">
         <is>
-          <t>PARTIAL FIT: this funder targets physical activity as an intervention for anxiety and depression. The org does psychoeducation and emotional wellness, not movement programming - a competitive application would need a genuine activity-based component, not a relabelling of existing workshops.</t>
+          <t>Reentry employment is a workable framing. Note this is the same corporate family as Champions in Action - a relationship built through one may help the other. Amount unpublished.</t>
         </is>
       </c>
     </row>
@@ -1827,21 +1827,21 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>JAMS Foundation NAFCM Mini-Grant Program</t>
+          <t>Job Opportunities for Building Success</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>JAMS Foundation</t>
+          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Private foundation</t>
+          <t>State / regional</t>
         </is>
       </c>
       <c r="E23" s="15" t="n">
-        <v>46441</v>
+        <v>46450</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -1854,22 +1854,22 @@
       </c>
       <c r="H23" s="10" t="n"/>
       <c r="I23" s="10" t="n">
-        <v>15000</v>
+        <v>1000000</v>
       </c>
       <c r="J23" s="11">
         <f>IF(AND(H23&lt;&gt;"",I23&lt;&gt;""),AVERAGE(H23:I23),IF(I23&lt;&gt;"",I23*$C$3,IF(H23&lt;&gt;"",H23,"")))</f>
         <v/>
       </c>
       <c r="K23" s="12" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="L23" s="11">
         <f>IF(OR(J23="",K23=""),"",J23*K23)</f>
         <v/>
       </c>
-      <c r="M23" s="18" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="M23" s="17" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="N23" s="14" t="n"/>
@@ -1877,7 +1877,7 @@
       <c r="P23" s="14" t="n"/>
       <c r="Q23" s="8" t="inlineStr">
         <is>
-          <t>ELIGIBILITY RISK: administered with the National Association for Community Mediation and generally aimed at NAFCM member community mediation centers. The org is not a mediation center. Anger management and healthy communication workshops map to the subject matter, but confirm whether non-member organizations can apply at all before spending time here.</t>
+          <t>Reentry employment framing works, but competitors are established workforce development agencies.</t>
         </is>
       </c>
     </row>
@@ -1887,12 +1887,12 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Citizens Philanthropic Foundation: Financial Empowerment</t>
+          <t>Family foundations (Scripps, Kim/Kayasa, Bernau, Scaife)</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Citizens Philanthropic Foundation</t>
+          <t>Various</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -1900,12 +1900,10 @@
           <t>Private foundation</t>
         </is>
       </c>
-      <c r="E24" s="15" t="n">
-        <v>46357</v>
-      </c>
+      <c r="E24" s="7" t="n"/>
       <c r="F24" s="7" t="inlineStr">
         <is>
-          <t>Pre-proposal</t>
+          <t>Rolling / 2027</t>
         </is>
       </c>
       <c r="G24" s="7">
@@ -1919,7 +1917,7 @@
         <v/>
       </c>
       <c r="K24" s="12" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="L24" s="11">
         <f>IF(OR(J24="",K24=""),"",J24*K24)</f>
@@ -1935,7 +1933,7 @@
       <c r="P24" s="14" t="n"/>
       <c r="Q24" s="8" t="inlineStr">
         <is>
-          <t>Weakest fit of the five: this track funds financial literacy and coaching, which the org does not currently deliver. Nearest deadline of the group, but would require standing up a service line rather than describing one.</t>
+          <t>Priorities unpublished; many small family foundations are effectively invitation-only. Pull Form 990s before writing - 15 min each tells you whether they accept unsolicited requests at all.</t>
         </is>
       </c>
     </row>
@@ -1945,21 +1943,21 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Second Chance Act - Family-Based SUD Treatment</t>
+          <t>Get Out and Get Active Grant</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>US DOJ, BJA</t>
+          <t>Anxiety &amp; Depression Initiative</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E25" s="15" t="n">
-        <v>46289</v>
+        <v>46504</v>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
@@ -1972,22 +1970,22 @@
       </c>
       <c r="H25" s="10" t="n"/>
       <c r="I25" s="10" t="n">
-        <v>1000000</v>
+        <v>10000</v>
       </c>
       <c r="J25" s="11">
         <f>IF(AND(H25&lt;&gt;"",I25&lt;&gt;""),AVERAGE(H25:I25),IF(I25&lt;&gt;"",I25*$C$3,IF(H25&lt;&gt;"",H25,"")))</f>
         <v/>
       </c>
       <c r="K25" s="12" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="L25" s="11">
         <f>IF(OR(J25="",K25=""),"",J25*K25)</f>
         <v/>
       </c>
-      <c r="M25" s="18" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="M25" s="17" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="N25" s="14" t="n"/>
@@ -1995,7 +1993,7 @@
       <c r="P25" s="14" t="n"/>
       <c r="Q25" s="8" t="inlineStr">
         <is>
-          <t>BEST MISSION FIT on the entire list. Barriers: national competition, 3x-budget award, and the 'treatment provider' question (org refers out to IOP rather than treating directly). Pursue as partner/sub-awardee.</t>
+          <t>PARTIAL FIT: this funder targets physical activity as an intervention for anxiety and depression. The org does psychoeducation and emotional wellness, not movement programming - a competitive application would need a genuine activity-based component, not a relabelling of existing workshops.</t>
         </is>
       </c>
     </row>
@@ -2005,25 +2003,25 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Second Chance Act - Reentry Education &amp; Employment</t>
+          <t>JAMS Foundation NAFCM Mini-Grant Program</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>US DOJ, BJA</t>
+          <t>JAMS Foundation</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E26" s="15" t="n">
-        <v>46289</v>
+        <v>46441</v>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>LOI</t>
         </is>
       </c>
       <c r="G26" s="7">
@@ -2032,14 +2030,14 @@
       </c>
       <c r="H26" s="10" t="n"/>
       <c r="I26" s="10" t="n">
-        <v>1000000</v>
+        <v>15000</v>
       </c>
       <c r="J26" s="11">
         <f>IF(AND(H26&lt;&gt;"",I26&lt;&gt;""),AVERAGE(H26:I26),IF(I26&lt;&gt;"",I26*$C$3,IF(H26&lt;&gt;"",H26,"")))</f>
         <v/>
       </c>
       <c r="K26" s="12" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="L26" s="11">
         <f>IF(OR(J26="",K26=""),"",J26*K26)</f>
@@ -2055,7 +2053,7 @@
       <c r="P26" s="14" t="n"/>
       <c r="Q26" s="8" t="inlineStr">
         <is>
-          <t>Federal reentry competitions draw established national providers with prior DOJ awards. Pursue as partner/sub-awardee.</t>
+          <t>ELIGIBILITY RISK: administered with the National Association for Community Mediation and generally aimed at NAFCM member community mediation centers. The org is not a mediation center. Anger management and healthy communication workshops map to the subject matter, but confirm whether non-member organizations can apply at all before spending time here.</t>
         </is>
       </c>
     </row>
@@ -2065,25 +2063,25 @@
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Project Grant</t>
+          <t>Citizens Philanthropic Foundation: Financial Empowerment</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>State Justice Institute</t>
+          <t>Citizens Philanthropic Foundation</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>Federal</t>
+          <t>Private foundation</t>
         </is>
       </c>
       <c r="E27" s="15" t="n">
-        <v>46327</v>
+        <v>46357</v>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Full</t>
+          <t>Pre-proposal</t>
         </is>
       </c>
       <c r="G27" s="7">
@@ -2091,15 +2089,13 @@
         <v/>
       </c>
       <c r="H27" s="10" t="n"/>
-      <c r="I27" s="10" t="n">
-        <v>300000</v>
-      </c>
+      <c r="I27" s="10" t="n"/>
       <c r="J27" s="11">
         <f>IF(AND(H27&lt;&gt;"",I27&lt;&gt;""),AVERAGE(H27:I27),IF(I27&lt;&gt;"",I27*$C$3,IF(H27&lt;&gt;"",H27,"")))</f>
         <v/>
       </c>
       <c r="K27" s="12" t="n">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
       <c r="L27" s="11">
         <f>IF(OR(J27="",K27=""),"",J27*K27)</f>
@@ -2115,7 +2111,7 @@
       <c r="P27" s="14" t="n"/>
       <c r="Q27" s="8" t="inlineStr">
         <is>
-          <t>SJI funds court systems. Realistic path is as named program partner on a court-led application - the recovery court relationship could support that.</t>
+          <t>Weakest fit of the five: this track funds financial literacy and coaching, which the org does not currently deliver. Nearest deadline of the group, but would require standing up a service line rather than describing one.</t>
         </is>
       </c>
     </row>
@@ -2125,25 +2121,25 @@
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>SNAP STEPS</t>
+          <t>Second Chance Act - Family-Based SUD Treatment</t>
         </is>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
+          <t>US DOJ, BJA</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="E28" s="15" t="n">
-        <v>46277</v>
+        <v>46289</v>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>LOI</t>
+          <t>Full</t>
         </is>
       </c>
       <c r="G28" s="7">
@@ -2152,20 +2148,22 @@
       </c>
       <c r="H28" s="10" t="n"/>
       <c r="I28" s="10" t="n">
-        <v>500000</v>
+        <v>1000000</v>
       </c>
       <c r="J28" s="11">
         <f>IF(AND(H28&lt;&gt;"",I28&lt;&gt;""),AVERAGE(H28:I28),IF(I28&lt;&gt;"",I28*$C$3,IF(H28&lt;&gt;"",H28,"")))</f>
         <v/>
       </c>
-      <c r="K28" s="12" t="n"/>
+      <c r="K28" s="12" t="n">
+        <v>0.06</v>
+      </c>
       <c r="L28" s="11">
         <f>IF(OR(J28="",K28=""),"",J28*K28)</f>
         <v/>
       </c>
-      <c r="M28" s="19" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="M28" s="18" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N28" s="14" t="n"/>
@@ -2173,7 +2171,7 @@
       <c r="P28" s="14" t="n"/>
       <c r="Q28" s="8" t="inlineStr">
         <is>
-          <t>VERIFY FIRST: near-term LOI. Overlap with reentry population is real but the org would need a workforce services track record.</t>
+          <t>BEST MISSION FIT on the entire list. Barriers: national competition, 3x-budget award, and the 'treatment provider' question (org refers out to IOP rather than treating directly). Pursue as partner/sub-awardee.</t>
         </is>
       </c>
     </row>
@@ -2183,21 +2181,21 @@
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Preventive Health Services Grant Program</t>
+          <t>Second Chance Act - Reentry Education &amp; Employment</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Health</t>
+          <t>US DOJ, BJA</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="E29" s="15" t="n">
-        <v>46343</v>
+        <v>46289</v>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
@@ -2210,20 +2208,22 @@
       </c>
       <c r="H29" s="10" t="n"/>
       <c r="I29" s="10" t="n">
-        <v>535000</v>
+        <v>1000000</v>
       </c>
       <c r="J29" s="11">
         <f>IF(AND(H29&lt;&gt;"",I29&lt;&gt;""),AVERAGE(H29:I29),IF(I29&lt;&gt;"",I29*$C$3,IF(H29&lt;&gt;"",H29,"")))</f>
         <v/>
       </c>
-      <c r="K29" s="12" t="n"/>
+      <c r="K29" s="12" t="n">
+        <v>0.05</v>
+      </c>
       <c r="L29" s="11">
         <f>IF(OR(J29="",K29=""),"",J29*K29)</f>
         <v/>
       </c>
-      <c r="M29" s="19" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="M29" s="18" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N29" s="14" t="n"/>
@@ -2231,7 +2231,7 @@
       <c r="P29" s="14" t="n"/>
       <c r="Q29" s="8" t="inlineStr">
         <is>
-          <t>VERIFY FIRST: confirm community nonprofits are eligible applicants rather than local health departments.</t>
+          <t>Federal reentry competitions draw established national providers with prior DOJ awards. Pursue as partner/sub-awardee.</t>
         </is>
       </c>
     </row>
@@ -2241,21 +2241,21 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Omnibus Eviction and Homelessness Prevention</t>
+          <t>Project Grant</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Community Affairs</t>
+          <t>State Justice Institute</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
-          <t>State / regional</t>
+          <t>Federal</t>
         </is>
       </c>
       <c r="E30" s="15" t="n">
-        <v>46358</v>
+        <v>46327</v>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -2267,19 +2267,23 @@
         <v/>
       </c>
       <c r="H30" s="10" t="n"/>
-      <c r="I30" s="10" t="n"/>
+      <c r="I30" s="10" t="n">
+        <v>300000</v>
+      </c>
       <c r="J30" s="11">
         <f>IF(AND(H30&lt;&gt;"",I30&lt;&gt;""),AVERAGE(H30:I30),IF(I30&lt;&gt;"",I30*$C$3,IF(H30&lt;&gt;"",H30,"")))</f>
         <v/>
       </c>
-      <c r="K30" s="12" t="n"/>
+      <c r="K30" s="12" t="n">
+        <v>0.05</v>
+      </c>
       <c r="L30" s="11">
         <f>IF(OR(J30="",K30=""),"",J30*K30)</f>
         <v/>
       </c>
-      <c r="M30" s="19" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="M30" s="18" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="N30" s="14" t="n"/>
@@ -2287,7 +2291,7 @@
       <c r="P30" s="14" t="n"/>
       <c r="Q30" s="8" t="inlineStr">
         <is>
-          <t>VERIFY FIRST: housing stability is adjacent to reentry wraparound; founder's lived experience with homelessness is relevant framing. Second RFP 2026-12-09.</t>
+          <t>SJI funds court systems. Realistic path is as named program partner on a court-led application - the recovery court relationship could support that.</t>
         </is>
       </c>
     </row>
@@ -2297,12 +2301,12 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Chronic Disease Prevention Grant</t>
+          <t>SNAP STEPS</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>NJ Dept. of Health</t>
+          <t>NJ Dept. of Labor &amp; Workforce Dev.</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
@@ -2311,7 +2315,7 @@
         </is>
       </c>
       <c r="E31" s="15" t="n">
-        <v>46379</v>
+        <v>46277</v>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
@@ -2324,7 +2328,7 @@
       </c>
       <c r="H31" s="10" t="n"/>
       <c r="I31" s="10" t="n">
-        <v>150000</v>
+        <v>500000</v>
       </c>
       <c r="J31" s="11">
         <f>IF(AND(H31&lt;&gt;"",I31&lt;&gt;""),AVERAGE(H31:I31),IF(I31&lt;&gt;"",I31*$C$3,IF(H31&lt;&gt;"",H31,"")))</f>
@@ -2345,45 +2349,217 @@
       <c r="P31" s="14" t="n"/>
       <c r="Q31" s="8" t="inlineStr">
         <is>
+          <t>VERIFY FIRST: near-term LOI. Overlap with reentry population is real but the org would need a workforce services track record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="46" customHeight="1">
+      <c r="A32" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Preventive Health Services Grant Program</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>NJ Dept. of Health</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E32" s="15" t="n">
+        <v>46343</v>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G32" s="7">
+        <f>IF(E32="","",E32-TODAY())</f>
+        <v/>
+      </c>
+      <c r="H32" s="10" t="n"/>
+      <c r="I32" s="10" t="n">
+        <v>535000</v>
+      </c>
+      <c r="J32" s="11">
+        <f>IF(AND(H32&lt;&gt;"",I32&lt;&gt;""),AVERAGE(H32:I32),IF(I32&lt;&gt;"",I32*$C$3,IF(H32&lt;&gt;"",H32,"")))</f>
+        <v/>
+      </c>
+      <c r="K32" s="12" t="n"/>
+      <c r="L32" s="11">
+        <f>IF(OR(J32="",K32=""),"",J32*K32)</f>
+        <v/>
+      </c>
+      <c r="M32" s="19" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N32" s="14" t="n"/>
+      <c r="O32" s="14" t="n"/>
+      <c r="P32" s="14" t="n"/>
+      <c r="Q32" s="8" t="inlineStr">
+        <is>
+          <t>VERIFY FIRST: confirm community nonprofits are eligible applicants rather than local health departments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="46" customHeight="1">
+      <c r="A33" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Omnibus Eviction and Homelessness Prevention</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>NJ Dept. of Community Affairs</t>
+        </is>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
+        <is>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="n">
+        <v>46358</v>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="G33" s="7">
+        <f>IF(E33="","",E33-TODAY())</f>
+        <v/>
+      </c>
+      <c r="H33" s="10" t="n"/>
+      <c r="I33" s="10" t="n"/>
+      <c r="J33" s="11">
+        <f>IF(AND(H33&lt;&gt;"",I33&lt;&gt;""),AVERAGE(H33:I33),IF(I33&lt;&gt;"",I33*$C$3,IF(H33&lt;&gt;"",H33,"")))</f>
+        <v/>
+      </c>
+      <c r="K33" s="12" t="n"/>
+      <c r="L33" s="11">
+        <f>IF(OR(J33="",K33=""),"",J33*K33)</f>
+        <v/>
+      </c>
+      <c r="M33" s="19" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N33" s="14" t="n"/>
+      <c r="O33" s="14" t="n"/>
+      <c r="P33" s="14" t="n"/>
+      <c r="Q33" s="8" t="inlineStr">
+        <is>
+          <t>VERIFY FIRST: housing stability is adjacent to reentry wraparound; founder's lived experience with homelessness is relevant framing. Second RFP 2026-12-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="46" customHeight="1">
+      <c r="A34" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Chronic Disease Prevention Grant</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>NJ Dept. of Health</t>
+        </is>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>State / regional</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="n">
+        <v>46379</v>
+      </c>
+      <c r="F34" s="7" t="inlineStr">
+        <is>
+          <t>LOI</t>
+        </is>
+      </c>
+      <c r="G34" s="7">
+        <f>IF(E34="","",E34-TODAY())</f>
+        <v/>
+      </c>
+      <c r="H34" s="10" t="n"/>
+      <c r="I34" s="10" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J34" s="11">
+        <f>IF(AND(H34&lt;&gt;"",I34&lt;&gt;""),AVERAGE(H34:I34),IF(I34&lt;&gt;"",I34*$C$3,IF(H34&lt;&gt;"",H34,"")))</f>
+        <v/>
+      </c>
+      <c r="K34" s="12" t="n"/>
+      <c r="L34" s="11">
+        <f>IF(OR(J34="",K34=""),"",J34*K34)</f>
+        <v/>
+      </c>
+      <c r="M34" s="19" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="N34" s="14" t="n"/>
+      <c r="O34" s="14" t="n"/>
+      <c r="P34" s="14" t="n"/>
+      <c r="Q34" s="8" t="inlineStr">
+        <is>
           <t>VERIFY FIRST: often targeted at diabetes/cardiovascular - confirm behavioral health is in scope this cycle.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="20" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="20" t="inlineStr">
         <is>
           <t>TOTAL PIPELINE</t>
         </is>
       </c>
-      <c r="J33" s="21">
-        <f>SUM(J5:J31)</f>
-        <v/>
-      </c>
-      <c r="L33" s="21">
-        <f>SUM(L5:L31)</f>
-        <v/>
-      </c>
-      <c r="M33" s="5" t="inlineStr">
+      <c r="J36" s="21">
+        <f>SUM(J5:J34)</f>
+        <v/>
+      </c>
+      <c r="L36" s="21">
+        <f>SUM(L5:L34)</f>
+        <v/>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
         <is>
           <t>&lt;- risk-weighted</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="28" customHeight="1">
-      <c r="B35" s="2" t="inlineStr">
+    <row r="38" ht="28" customHeight="1">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Expected Value = Planning Amount x Est. Win %. It is the risk-weighted worth of pursuing an item, NOT a forecast of what you will receive. Sorting by it gives a different order than sorting by likelihood - both are worth looking at.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:Q31"/>
+  <autoFilter ref="A4:Q34"/>
   <mergeCells count="2">
     <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="B35:Q35"/>
+    <mergeCell ref="B38:Q38"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="N5:N31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N5:N34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,Researching,Drafting,Submitted,Awarded,Declined,Skipped"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>